<commit_message>
Added a new error handling function, lecturers can now select the week they want to get attendance for. And also edit the attendace excel sheet
</commit_message>
<xml_diff>
--- a/Python/Attendance.xlsx
+++ b/Python/Attendance.xlsx
@@ -1,38 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/abbf0957561ee885/Desktop/RFID_Attendance_System/RFID_Attendance_System-SDG4/Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="11_F25DC773A252ABDACC1048C9F99957EE5BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{066B2F51-23A3-4E1E-9CBD-93C7309CAE5D}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="11_2B59D2BFD310DEB22341BF904D1510344D078C22" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54DA08DA-C80E-43DF-BD86-13CF1CA2F2C0}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>RFID_UID</t>
   </si>
   <si>
-    <t>Attendance</t>
-  </si>
-  <si>
     <t>Student_ID</t>
   </si>
   <si>
@@ -52,6 +44,51 @@
   </si>
   <si>
     <t>Foday Kamara</t>
+  </si>
+  <si>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Week 2</t>
+  </si>
+  <si>
+    <t>Week 3</t>
+  </si>
+  <si>
+    <t>Week 4</t>
+  </si>
+  <si>
+    <t>Week 5</t>
+  </si>
+  <si>
+    <t>Week 6</t>
+  </si>
+  <si>
+    <t>Week 7</t>
+  </si>
+  <si>
+    <t>Week 8</t>
+  </si>
+  <si>
+    <t>Week 9</t>
+  </si>
+  <si>
+    <t>Week 10</t>
+  </si>
+  <si>
+    <t>Week 11</t>
+  </si>
+  <si>
+    <t>Week 12</t>
+  </si>
+  <si>
+    <t>Week 13</t>
+  </si>
+  <si>
+    <t>Week 14</t>
+  </si>
+  <si>
+    <t>Week 15</t>
   </si>
 </sst>
 </file>
@@ -67,14 +104,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Tahoma"/>
+      <sz val="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Tahoma"/>
       <family val="2"/>
@@ -117,7 +154,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -128,7 +165,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -138,6 +175,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -151,44 +192,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -215,15 +256,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -250,7 +290,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -262,209 +301,415 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" customWidth="1"/>
-    <col min="2" max="2" width="19.44140625" customWidth="1"/>
-    <col min="3" max="3" width="31.5546875" customWidth="1"/>
-    <col min="4" max="4" width="20.77734375" customWidth="1"/>
+    <col min="1" max="2" width="15.21875" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" customWidth="1"/>
+    <col min="4" max="4" width="20.5546875" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" customWidth="1"/>
+    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="9" max="9" width="15.21875" customWidth="1"/>
+    <col min="10" max="10" width="13.77734375" customWidth="1"/>
+    <col min="11" max="11" width="16.21875" customWidth="1"/>
+    <col min="12" max="12" width="11.6640625" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="12.109375" customWidth="1"/>
+    <col min="15" max="15" width="14.33203125" customWidth="1"/>
+    <col min="16" max="16" width="16" customWidth="1"/>
+    <col min="17" max="17" width="10.88671875" customWidth="1"/>
+    <col min="18" max="18" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
+      <c r="B2" s="1">
+        <v>905005656</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1">
+        <v>0</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0</v>
+      </c>
+      <c r="N2" s="1">
+        <v>0</v>
+      </c>
+      <c r="O2" s="1">
+        <v>0</v>
+      </c>
+      <c r="P2" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>0</v>
+      </c>
+      <c r="R2" s="1">
+        <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2">
-        <v>905005656</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="2">
+      <c r="B3" s="1">
+        <v>905005267</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0</v>
+      </c>
+      <c r="L3" s="1">
+        <v>0</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0</v>
+      </c>
+      <c r="N3" s="1">
+        <v>0</v>
+      </c>
+      <c r="O3" s="1">
+        <v>0</v>
+      </c>
+      <c r="P3" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>0</v>
+      </c>
+      <c r="R3" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="2">
-        <v>905005267</v>
-      </c>
-      <c r="C3" s="2" t="s">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0</v>
+      </c>
+      <c r="L4" s="1">
+        <v>0</v>
+      </c>
+      <c r="M4" s="1">
+        <v>0</v>
+      </c>
+      <c r="N4" s="1">
+        <v>0</v>
+      </c>
+      <c r="O4" s="1">
+        <v>0</v>
+      </c>
+      <c r="P4" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>0</v>
+      </c>
+      <c r="R4" s="1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reseted the excel database, everything should be null
</commit_message>
<xml_diff>
--- a/Python/Attendance.xlsx
+++ b/Python/Attendance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/abbf0957561ee885/Desktop/RFID_Attendance_System/RFID_Attendance_System-SDG4/Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59D2BFD330536AE1E0CEF050C9E0344F2FF452" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{851DF4E1-65FB-4430-9FD8-3240F0E0FA6B}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_2B59D2BFD330536AE1E0CEF050C9E0344F2FF452" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B070658-906D-4FC9-8D98-22860CC4A3BD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -135,6 +135,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -483,10 +487,10 @@
         <v>16</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -530,10 +534,10 @@
         <v>18</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -574,10 +578,10 @@
         <v>20</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4">
         <v>0</v>

</xml_diff>

<commit_message>
Adding the binary status 0-absent, 1-present. Also fix bugs that was making the lED not to blink
</commit_message>
<xml_diff>
--- a/Python/Attendance.xlsx
+++ b/Python/Attendance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/abbf0957561ee885/Desktop/RFID_Attendance_System/RFID_Attendance_System-SDG4/Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_2B59D2BFD370596B19E3DBF0509E28B16E51E3DC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{918D1A36-70B8-4882-B39C-EC68C3AF0633}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="11_2B59D2BFD320592C6121CEF050A458B74DBBE3F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB94EED2-4616-4555-8312-F0420F54D804}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>RFID_UID</t>
   </si>
@@ -136,7 +136,7 @@
     <t>Rayan Martin Turay</t>
   </si>
   <si>
-    <t>FA50CA35</t>
+    <t>4FA50CA35</t>
   </si>
   <si>
     <t>Abdul Karim Koroma</t>
@@ -146,16 +146,31 @@
   </si>
   <si>
     <t>Foday Kamara</t>
+  </si>
+  <si>
+    <t>Week3_Departure</t>
+  </si>
+  <si>
+    <t>Week3_Status</t>
+  </si>
+  <si>
+    <t>Week4_Arrival</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -489,13 +504,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AJ4"/>
+  <dimension ref="A1:AM4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -527,85 +542,94 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
+        <v>42</v>
+      </c>
+      <c r="L1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1" t="s">
+        <v>44</v>
+      </c>
+      <c r="N1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="P1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="Q1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="R1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="S1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="T1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="U1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="V1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="W1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="X1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="Y1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="Z1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="AA1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="AB1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AC1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AD1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AE1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AF1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AG1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AH1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AI1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AJ1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AK1" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AL1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AM1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>36</v>
       </c>
@@ -615,8 +639,44 @@
       <c r="C2" t="s">
         <v>37</v>
       </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AG2">
+        <v>0</v>
+      </c>
+      <c r="AJ2">
+        <v>0</v>
+      </c>
+      <c r="AM2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -626,8 +686,44 @@
       <c r="C3" t="s">
         <v>39</v>
       </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AG3">
+        <v>0</v>
+      </c>
+      <c r="AJ3">
+        <v>0</v>
+      </c>
+      <c r="AM3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>40</v>
       </c>
@@ -637,8 +733,45 @@
       <c r="C4" t="s">
         <v>41</v>
       </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AG4">
+        <v>0</v>
+      </c>
+      <c r="AJ4">
+        <v>0</v>
+      </c>
+      <c r="AM4">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>